<commit_message>
chore(Proceso_cierre): actualizar referencia TC_mensual y diccionario_puntos (cierre 2026-09)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XMY2PbC44X7KVp1NjZNS2h
</commit_message>
<xml_diff>
--- a/Proceso_cierre/referencia/diccionario_puntos.xlsx
+++ b/Proceso_cierre/referencia/diccionario_puntos.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="305">
   <si>
     <t>id</t>
   </si>
@@ -430,6 +430,9 @@
     <t>C_BC_PL_WE</t>
   </si>
   <si>
+    <t>C_BC_EX_WE</t>
+  </si>
+  <si>
     <t>General points</t>
   </si>
   <si>
@@ -725,6 +728,9 @@
   </si>
   <si>
     <t>C_BC_PLATINUM_WELCOME</t>
+  </si>
+  <si>
+    <t>C_BC_EXTRA_WELCOME</t>
   </si>
   <si>
     <t>Bonus points</t>
@@ -922,6 +928,9 @@
   </si>
   <si>
     <t>Puntos bienvenida PLATINUM BDB</t>
+  </si>
+  <si>
+    <t>Puntos bienvenida extra por grupo BDB</t>
   </si>
 </sst>
 </file>
@@ -1253,7 +1262,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R121"/>
+  <dimension ref="A1:R122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
@@ -1320,10 +1329,10 @@
         <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -1352,10 +1361,10 @@
         <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
@@ -1384,10 +1393,10 @@
         <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -1416,10 +1425,10 @@
         <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
@@ -1451,10 +1460,10 @@
         <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
@@ -1486,10 +1495,10 @@
         <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
@@ -1521,10 +1530,10 @@
         <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
@@ -1556,10 +1565,10 @@
         <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
@@ -1591,10 +1600,10 @@
         <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -1626,10 +1635,10 @@
         <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E11" t="b">
         <v>1</v>
@@ -1661,10 +1670,10 @@
         <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E12" t="b">
         <v>1</v>
@@ -1696,10 +1705,10 @@
         <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E13" t="b">
         <v>1</v>
@@ -1731,10 +1740,10 @@
         <v>30</v>
       </c>
       <c r="C14" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D14" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E14" t="b">
         <v>1</v>
@@ -1766,10 +1775,10 @@
         <v>31</v>
       </c>
       <c r="C15" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D15" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E15" t="b">
         <v>1</v>
@@ -1801,10 +1810,10 @@
         <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D16" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E16" t="b">
         <v>1</v>
@@ -1836,10 +1845,10 @@
         <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D17" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E17" t="b">
         <v>1</v>
@@ -1871,10 +1880,10 @@
         <v>34</v>
       </c>
       <c r="C18" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D18" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E18" t="b">
         <v>1</v>
@@ -1906,10 +1915,10 @@
         <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D19" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E19" t="b">
         <v>1</v>
@@ -1941,10 +1950,10 @@
         <v>36</v>
       </c>
       <c r="C20" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D20" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E20" t="b">
         <v>1</v>
@@ -1976,10 +1985,10 @@
         <v>37</v>
       </c>
       <c r="C21" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D21" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E21" t="b">
         <v>1</v>
@@ -2011,10 +2020,10 @@
         <v>38</v>
       </c>
       <c r="C22" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D22" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E22" t="b">
         <v>1</v>
@@ -2046,10 +2055,10 @@
         <v>39</v>
       </c>
       <c r="C23" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D23" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E23" t="b">
         <v>1</v>
@@ -2081,10 +2090,10 @@
         <v>40</v>
       </c>
       <c r="C24" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D24" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E24" t="b">
         <v>1</v>
@@ -2116,7 +2125,7 @@
         <v>41</v>
       </c>
       <c r="C25" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E25" t="b">
         <v>1</v>
@@ -2148,10 +2157,10 @@
         <v>42</v>
       </c>
       <c r="C26" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D26" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E26" t="b">
         <v>1</v>
@@ -2183,10 +2192,10 @@
         <v>43</v>
       </c>
       <c r="C27" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D27" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E27" t="b">
         <v>1</v>
@@ -2218,10 +2227,10 @@
         <v>44</v>
       </c>
       <c r="C28" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D28" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E28" t="b">
         <v>1</v>
@@ -2253,10 +2262,10 @@
         <v>45</v>
       </c>
       <c r="C29" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D29" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E29" t="b">
         <v>1</v>
@@ -2288,10 +2297,10 @@
         <v>46</v>
       </c>
       <c r="C30" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D30" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E30" t="b">
         <v>1</v>
@@ -2323,10 +2332,10 @@
         <v>47</v>
       </c>
       <c r="C31" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D31" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E31" t="b">
         <v>1</v>
@@ -2358,10 +2367,10 @@
         <v>48</v>
       </c>
       <c r="C32" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D32" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E32" t="b">
         <v>1</v>
@@ -2393,10 +2402,10 @@
         <v>49</v>
       </c>
       <c r="C33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E33" t="b">
         <v>1</v>
@@ -2428,10 +2437,10 @@
         <v>50</v>
       </c>
       <c r="C34" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D34" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E34" t="b">
         <v>1</v>
@@ -2463,7 +2472,7 @@
         <v>51</v>
       </c>
       <c r="C35" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E35" t="b">
         <v>1</v>
@@ -2492,10 +2501,10 @@
         <v>52</v>
       </c>
       <c r="C36" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D36" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E36" t="b">
         <v>1</v>
@@ -2524,10 +2533,10 @@
         <v>53</v>
       </c>
       <c r="C37" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D37" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E37" t="b">
         <v>1</v>
@@ -2556,10 +2565,10 @@
         <v>54</v>
       </c>
       <c r="C38" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D38" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E38" t="b">
         <v>1</v>
@@ -2588,10 +2597,10 @@
         <v>55</v>
       </c>
       <c r="C39" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D39" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E39" t="b">
         <v>1</v>
@@ -2620,10 +2629,10 @@
         <v>56</v>
       </c>
       <c r="C40" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D40" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E40" t="b">
         <v>1</v>
@@ -2652,10 +2661,10 @@
         <v>57</v>
       </c>
       <c r="C41" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D41" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E41" t="b">
         <v>1</v>
@@ -2684,10 +2693,10 @@
         <v>58</v>
       </c>
       <c r="C42" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D42" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E42" t="b">
         <v>1</v>
@@ -2716,10 +2725,10 @@
         <v>59</v>
       </c>
       <c r="C43" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D43" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E43" t="b">
         <v>1</v>
@@ -2748,10 +2757,10 @@
         <v>60</v>
       </c>
       <c r="C44" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D44" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E44" t="b">
         <v>1</v>
@@ -2780,10 +2789,10 @@
         <v>61</v>
       </c>
       <c r="C45" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D45" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E45" t="b">
         <v>1</v>
@@ -2812,10 +2821,10 @@
         <v>62</v>
       </c>
       <c r="C46" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D46" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E46" t="b">
         <v>1</v>
@@ -2844,7 +2853,7 @@
         <v>63</v>
       </c>
       <c r="C47" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E47" t="b">
         <v>1</v>
@@ -2873,10 +2882,10 @@
         <v>64</v>
       </c>
       <c r="C48" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D48" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E48" t="b">
         <v>1</v>
@@ -2905,10 +2914,10 @@
         <v>65</v>
       </c>
       <c r="C49" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D49" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E49" t="b">
         <v>1</v>
@@ -2937,7 +2946,7 @@
         <v>66</v>
       </c>
       <c r="C50" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E50" t="b">
         <v>1</v>
@@ -2975,7 +2984,7 @@
         <v>67</v>
       </c>
       <c r="C51" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E51" t="b">
         <v>1</v>
@@ -3013,7 +3022,7 @@
         <v>68</v>
       </c>
       <c r="C52" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E52" t="b">
         <v>1</v>
@@ -3051,7 +3060,7 @@
         <v>69</v>
       </c>
       <c r="C53" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E53" t="b">
         <v>1</v>
@@ -3089,7 +3098,7 @@
         <v>70</v>
       </c>
       <c r="C54" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E54" t="b">
         <v>1</v>
@@ -3127,7 +3136,7 @@
         <v>71</v>
       </c>
       <c r="C55" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E55" t="b">
         <v>1</v>
@@ -3165,7 +3174,7 @@
         <v>72</v>
       </c>
       <c r="C56" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E56" t="b">
         <v>1</v>
@@ -3203,7 +3212,7 @@
         <v>73</v>
       </c>
       <c r="C57" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E57" t="b">
         <v>1</v>
@@ -3241,7 +3250,7 @@
         <v>74</v>
       </c>
       <c r="C58" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E58" t="b">
         <v>1</v>
@@ -3279,7 +3288,7 @@
         <v>75</v>
       </c>
       <c r="C59" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E59" t="b">
         <v>1</v>
@@ -3317,7 +3326,7 @@
         <v>76</v>
       </c>
       <c r="C60" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E60" t="b">
         <v>1</v>
@@ -3355,7 +3364,7 @@
         <v>77</v>
       </c>
       <c r="C61" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E61" t="b">
         <v>1</v>
@@ -3393,7 +3402,7 @@
         <v>78</v>
       </c>
       <c r="C62" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E62" t="b">
         <v>1</v>
@@ -3422,10 +3431,10 @@
         <v>79</v>
       </c>
       <c r="C63" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D63" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E63" t="b">
         <v>1</v>
@@ -3454,7 +3463,7 @@
         <v>80</v>
       </c>
       <c r="C64" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E64" t="b">
         <v>1</v>
@@ -3483,10 +3492,10 @@
         <v>81</v>
       </c>
       <c r="C65" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D65" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E65" t="b">
         <v>1</v>
@@ -3518,7 +3527,7 @@
         <v>82</v>
       </c>
       <c r="D66" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E66" t="b">
         <v>1</v>
@@ -3547,10 +3556,10 @@
         <v>83</v>
       </c>
       <c r="C67" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D67" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E67" t="b">
         <v>1</v>
@@ -3582,7 +3591,7 @@
         <v>84</v>
       </c>
       <c r="D68" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E68" t="b">
         <v>1</v>
@@ -3611,10 +3620,10 @@
         <v>85</v>
       </c>
       <c r="C69" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D69" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E69" t="b">
         <v>1</v>
@@ -3646,10 +3655,10 @@
         <v>86</v>
       </c>
       <c r="C70" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D70" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E70" t="b">
         <v>1</v>
@@ -3681,10 +3690,10 @@
         <v>87</v>
       </c>
       <c r="C71" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D71" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E71" t="b">
         <v>1</v>
@@ -3716,10 +3725,10 @@
         <v>88</v>
       </c>
       <c r="C72" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D72" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E72" t="b">
         <v>1</v>
@@ -3751,10 +3760,10 @@
         <v>89</v>
       </c>
       <c r="C73" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D73" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E73" t="b">
         <v>1</v>
@@ -3786,10 +3795,10 @@
         <v>90</v>
       </c>
       <c r="C74" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D74" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E74" t="b">
         <v>1</v>
@@ -3821,10 +3830,10 @@
         <v>91</v>
       </c>
       <c r="C75" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D75" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E75" t="b">
         <v>1</v>
@@ -3856,10 +3865,10 @@
         <v>92</v>
       </c>
       <c r="C76" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D76" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E76" t="b">
         <v>1</v>
@@ -3891,10 +3900,10 @@
         <v>93</v>
       </c>
       <c r="C77" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D77" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E77" t="b">
         <v>1</v>
@@ -3926,10 +3935,10 @@
         <v>94</v>
       </c>
       <c r="C78" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D78" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E78" t="b">
         <v>1</v>
@@ -3958,10 +3967,10 @@
         <v>95</v>
       </c>
       <c r="C79" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D79" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E79" t="b">
         <v>1</v>
@@ -4022,7 +4031,7 @@
         <v>97</v>
       </c>
       <c r="D81" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E81" t="b">
         <v>1</v>
@@ -4138,10 +4147,10 @@
         <v>101</v>
       </c>
       <c r="C85" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D85" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E85" t="b">
         <v>1</v>
@@ -4199,7 +4208,7 @@
         <v>103</v>
       </c>
       <c r="C87" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E87" t="b">
         <v>1</v>
@@ -4231,7 +4240,7 @@
         <v>104</v>
       </c>
       <c r="D88" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E88" t="b">
         <v>1</v>
@@ -4260,10 +4269,10 @@
         <v>105</v>
       </c>
       <c r="C89" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D89" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E89" t="b">
         <v>1</v>
@@ -4292,10 +4301,10 @@
         <v>106</v>
       </c>
       <c r="C90" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D90" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E90" t="b">
         <v>1</v>
@@ -4327,7 +4336,7 @@
         <v>107</v>
       </c>
       <c r="D91" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E91" t="b">
         <v>1</v>
@@ -4356,10 +4365,10 @@
         <v>108</v>
       </c>
       <c r="C92" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D92" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E92" t="b">
         <v>1</v>
@@ -4388,10 +4397,10 @@
         <v>109</v>
       </c>
       <c r="C93" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D93" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E93" t="b">
         <v>1</v>
@@ -4420,10 +4429,10 @@
         <v>110</v>
       </c>
       <c r="C94" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D94" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E94" t="b">
         <v>1</v>
@@ -4455,7 +4464,7 @@
         <v>111</v>
       </c>
       <c r="D95" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="E95" t="b">
         <v>1</v>
@@ -4484,10 +4493,10 @@
         <v>112</v>
       </c>
       <c r="C96" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D96" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E96" t="b">
         <v>1</v>
@@ -4516,10 +4525,10 @@
         <v>113</v>
       </c>
       <c r="C97" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D97" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E97" t="b">
         <v>1</v>
@@ -4551,7 +4560,7 @@
         <v>114</v>
       </c>
       <c r="D98" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E98" t="b">
         <v>1</v>
@@ -4583,7 +4592,7 @@
         <v>115</v>
       </c>
       <c r="D99" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E99" t="b">
         <v>1</v>
@@ -4612,10 +4621,10 @@
         <v>116</v>
       </c>
       <c r="C100" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D100" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E100" t="b">
         <v>1</v>
@@ -4644,10 +4653,10 @@
         <v>117</v>
       </c>
       <c r="C101" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D101" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E101" t="b">
         <v>1</v>
@@ -4679,7 +4688,7 @@
         <v>118</v>
       </c>
       <c r="D102" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E102" t="b">
         <v>1</v>
@@ -4711,7 +4720,7 @@
         <v>119</v>
       </c>
       <c r="D103" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E103" t="b">
         <v>1</v>
@@ -4743,7 +4752,7 @@
         <v>120</v>
       </c>
       <c r="D104" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E104" t="b">
         <v>1</v>
@@ -4775,7 +4784,7 @@
         <v>121</v>
       </c>
       <c r="D105" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E105" t="b">
         <v>1</v>
@@ -4807,7 +4816,7 @@
         <v>122</v>
       </c>
       <c r="D106" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E106" t="b">
         <v>1</v>
@@ -4839,7 +4848,7 @@
         <v>123</v>
       </c>
       <c r="D107" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="E107" t="b">
         <v>1</v>
@@ -4871,7 +4880,7 @@
         <v>124</v>
       </c>
       <c r="D108" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E108" t="b">
         <v>1</v>
@@ -4900,10 +4909,10 @@
         <v>125</v>
       </c>
       <c r="C109" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D109" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="E109" t="b">
         <v>1</v>
@@ -4935,10 +4944,10 @@
         <v>126</v>
       </c>
       <c r="C110" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D110" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E110" t="b">
         <v>1</v>
@@ -4970,10 +4979,10 @@
         <v>127</v>
       </c>
       <c r="C111" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D111" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E111" t="b">
         <v>1</v>
@@ -5005,10 +5014,10 @@
         <v>128</v>
       </c>
       <c r="C112" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D112" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E112" t="b">
         <v>1</v>
@@ -5040,10 +5049,10 @@
         <v>129</v>
       </c>
       <c r="C113" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D113" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E113" t="b">
         <v>1</v>
@@ -5075,10 +5084,10 @@
         <v>130</v>
       </c>
       <c r="C114" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D114" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E114" t="b">
         <v>1</v>
@@ -5113,7 +5122,7 @@
         <v>131</v>
       </c>
       <c r="D115" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="E115" t="b">
         <v>1</v>
@@ -5142,10 +5151,10 @@
         <v>132</v>
       </c>
       <c r="C116" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D116" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E116" t="b">
         <v>1</v>
@@ -5177,10 +5186,10 @@
         <v>133</v>
       </c>
       <c r="C117" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D117" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E117" t="b">
         <v>1</v>
@@ -5212,10 +5221,10 @@
         <v>134</v>
       </c>
       <c r="C118" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D118" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E118" t="b">
         <v>1</v>
@@ -5247,10 +5256,10 @@
         <v>135</v>
       </c>
       <c r="C119" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D119" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E119" t="b">
         <v>1</v>
@@ -5282,10 +5291,10 @@
         <v>136</v>
       </c>
       <c r="C120" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D120" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E120" t="b">
         <v>1</v>
@@ -5317,10 +5326,10 @@
         <v>137</v>
       </c>
       <c r="C121" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D121" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E121" t="b">
         <v>1</v>
@@ -5341,297 +5350,45 @@
         <v>119</v>
       </c>
       <c r="P121" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:16">
+      <c r="A122">
+        <v>3301</v>
+      </c>
+      <c r="B122" t="s">
+        <v>138</v>
+      </c>
+      <c r="C122" t="s">
+        <v>238</v>
+      </c>
+      <c r="D122" t="s">
+        <v>304</v>
+      </c>
+      <c r="E122" t="b">
+        <v>1</v>
+      </c>
+      <c r="F122">
+        <v>18</v>
+      </c>
+      <c r="H122" t="b">
+        <v>0</v>
+      </c>
+      <c r="I122" t="b">
+        <v>1</v>
+      </c>
+      <c r="J122" t="b">
+        <v>0</v>
+      </c>
+      <c r="N122">
+        <v>121</v>
+      </c>
+      <c r="P122" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101003CABB80693E2184BB67E2D9B1AEB302B" ma:contentTypeVersion="18" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="ae7fc125f0922bd81aa9fff759d982e7">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7c7b89f8-bfb0-4f6d-aa93-a7df2a1a6821" xmlns:ns3="943ab931-17a6-4e89-bad1-eed902ff4899" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9739e70e4b5540fc937fb84f0a71f128" ns2:_="" ns3:_="">
-    <xsd:import namespace="7c7b89f8-bfb0-4f6d-aa93-a7df2a1a6821"/>
-    <xsd:import namespace="943ab931-17a6-4e89-bad1-eed902ff4899"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="7c7b89f8-bfb0-4f6d-aa93-a7df2a1a6821" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="10" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="11" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="12" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="13" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="16" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="21" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="9f319c45-f596-4753-90b2-770d30d74f6f" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="23" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="24" nillable="true" ma:displayName="Location" ma:description="" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="943ab931-17a6-4e89-bad1-eed902ff4899" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="17" nillable="true" ma:displayName="Compartido con" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="18" nillable="true" ma:displayName="Detalles de uso compartido" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="22" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{7e81ccc8-5e4f-4a27-98b9-fd6f38cc8f91}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="943ab931-17a6-4e89-bad1-eed902ff4899">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7c7b89f8-bfb0-4f6d-aa93-a7df2a1a6821">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="943ab931-17a6-4e89-bad1-eed902ff4899" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C15415EB-9E24-4F78-AD46-B84425EB19E0}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D164A866-B1F7-4231-96B6-F2C39936619F}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C63825AE-D3C6-4B1E-AF66-CE4D12C61257}"/>
 </file>
</xml_diff>